<commit_message>
Dashboard: trailing 6-month churn, avg stay, churn-based LTV
Churned clients come from the monthly metrics — the one record that goes
back before the projects were loaded — divided by a new Active Clients
metric entered alongside them, falling back to the accounts with a signed
retainer that month when it was left blank. The Churn card shows the
monthly rate, the implied average stay, clients lost in the window, and
how many churned accounts left within three months (from project end
dates, per account so a re-signed client isn't counted twice).

Avg Client Lifetime is now avg monthly value ÷ churn, the standard form,
and the Growth Projection seeds its churn % from the same rate.

Active Clients is accepted by the metrics table, bulk paste, and the
intake template. The column was added to the live DB with a single
ADD COLUMN rather than db:push.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Client-Intake-Template.xlsx
+++ b/public/Client-Intake-Template.xlsx
@@ -540,7 +540,6 @@
           <t>Your name</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -548,7 +547,6 @@
           <t>Agency name</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -556,7 +554,6 @@
           <t>Email</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -685,7 +682,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:K3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -698,6 +695,7 @@
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="15" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -758,6 +756,11 @@
           <t>Marketing Spend</t>
         </is>
       </c>
+      <c r="K2" s="4" t="inlineStr">
+        <is>
+          <t>Active Clients</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
@@ -791,6 +794,9 @@
       </c>
       <c r="J3" s="5" t="n">
         <v>1500</v>
+      </c>
+      <c r="K3" s="5" t="n">
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>